<commit_message>
Update MLB weather 2026-09-04 02:54 PM PT
</commit_message>
<xml_diff>
--- a/mlb_weather_professional_v5_2026_09_04.xlsx
+++ b/mlb_weather_professional_v5_2026_09_04.xlsx
@@ -713,21 +713,21 @@
     <t>FIRST RUN</t>
   </si>
   <si>
+    <t>IMPROVING</t>
+  </si>
+  <si>
     <t>STEADY</t>
   </si>
   <si>
     <t>WORSENING RAPIDLY</t>
   </si>
   <si>
-    <t>IMPROVING</t>
+    <t>WORSENING</t>
   </si>
   <si>
     <t>IMPROVING RAPIDLY</t>
   </si>
   <si>
-    <t>WORSENING</t>
-  </si>
-  <si>
     <t>MODERATE</t>
   </si>
   <si>
@@ -740,52 +740,52 @@
     <t>MEDIUM</t>
   </si>
   <si>
-    <t>2026-09-04 02:45:26 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:45:31 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:45:36 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:45:42 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:45:48 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:45:53 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:45:59 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:46:04 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:46:10 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:46:16 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:46:17 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:46:23 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:46:28 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:46:33 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:46:39 PM PDT</t>
-  </si>
-  <si>
-    <t>2026-09-04 02:46:44 PM PDT</t>
+    <t>2026-09-04 02:52:37 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:52:42 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:52:47 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:52:53 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:52:58 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:03 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:08 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:13 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:18 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:23 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:24 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:29 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:34 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:39 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:44 PM PDT</t>
+  </si>
+  <si>
+    <t>2026-09-04 02:53:49 PM PDT</t>
   </si>
   <si>
     <t>Period</t>
@@ -1265,52 +1265,52 @@
     <t>10:10 PM PDT</t>
   </si>
   <si>
-    <t>2026-09-04 21:45:26 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:45:31 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:45:36 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:45:42 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:45:48 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:45:53 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:45:59 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:46:04 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:46:10 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:46:16 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:46:17 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:46:23 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:46:28 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:46:33 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:46:39 UTC</t>
-  </si>
-  <si>
-    <t>2026-09-04 21:46:44 UTC</t>
+    <t>2026-09-04 21:52:37 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:52:42 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:52:47 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:52:53 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:52:58 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:03 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:08 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:13 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:18 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:23 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:24 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:29 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:34 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:39 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:44 UTC</t>
+  </si>
+  <si>
+    <t>2026-09-04 21:53:49 UTC</t>
   </si>
   <si>
     <t>2026-09-04T19:47:12+00:00</t>
@@ -2359,7 +2359,7 @@
         <v>239</v>
       </c>
       <c r="BO2">
-        <v>118.2</v>
+        <v>125.4</v>
       </c>
       <c r="BP2">
         <v>5</v>
@@ -2535,7 +2535,7 @@
         <v>230</v>
       </c>
       <c r="BG3">
-        <v>0.4</v>
+        <v>2.5</v>
       </c>
       <c r="BH3">
         <v>-0.54</v>
@@ -2559,7 +2559,7 @@
         <v>240</v>
       </c>
       <c r="BO3">
-        <v>3.4</v>
+        <v>10.6</v>
       </c>
       <c r="BP3">
         <v>5</v>
@@ -2732,10 +2732,10 @@
         <v>70.8</v>
       </c>
       <c r="BF4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="BG4">
-        <v>-1.1</v>
+        <v>-1.3</v>
       </c>
       <c r="BH4">
         <v>-0.21</v>
@@ -2759,7 +2759,7 @@
         <v>241</v>
       </c>
       <c r="BO4">
-        <v>95.5</v>
+        <v>102.7</v>
       </c>
       <c r="BP4">
         <v>5</v>
@@ -2932,7 +2932,7 @@
         <v>85.2</v>
       </c>
       <c r="BF5" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="BG5">
         <v>0.9</v>
@@ -2959,7 +2959,7 @@
         <v>242</v>
       </c>
       <c r="BO5">
-        <v>78.5</v>
+        <v>85.7</v>
       </c>
       <c r="BP5">
         <v>5</v>
@@ -3132,10 +3132,10 @@
         <v>66.59999999999999</v>
       </c>
       <c r="BF6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="BG6">
-        <v>0.7</v>
+        <v>0.3</v>
       </c>
       <c r="BH6">
         <v>0.16</v>
@@ -3159,7 +3159,7 @@
         <v>243</v>
       </c>
       <c r="BO6">
-        <v>52.1</v>
+        <v>59.2</v>
       </c>
       <c r="BP6">
         <v>5</v>
@@ -3332,10 +3332,10 @@
         <v>51.7</v>
       </c>
       <c r="BF7" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="BG7">
-        <v>-5.3</v>
+        <v>-5.6</v>
       </c>
       <c r="BH7">
         <v>-0.5600000000000001</v>
@@ -3359,7 +3359,7 @@
         <v>244</v>
       </c>
       <c r="BO7">
-        <v>205.7</v>
+        <v>212.9</v>
       </c>
       <c r="BP7">
         <v>5</v>
@@ -3532,10 +3532,10 @@
         <v>83.7</v>
       </c>
       <c r="BF8" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="BG8">
-        <v>-4.1</v>
+        <v>-3.5</v>
       </c>
       <c r="BH8">
         <v>-0.49</v>
@@ -3559,7 +3559,7 @@
         <v>245</v>
       </c>
       <c r="BO8">
-        <v>104.2</v>
+        <v>111.4</v>
       </c>
       <c r="BP8">
         <v>5</v>
@@ -3732,10 +3732,10 @@
         <v>86.09999999999999</v>
       </c>
       <c r="BF9" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="BG9">
-        <v>-5.8</v>
+        <v>-4.9</v>
       </c>
       <c r="BH9">
         <v>-0.29</v>
@@ -3759,7 +3759,7 @@
         <v>246</v>
       </c>
       <c r="BO9">
-        <v>118.9</v>
+        <v>126</v>
       </c>
       <c r="BP9">
         <v>5</v>
@@ -3932,10 +3932,10 @@
         <v>69.7</v>
       </c>
       <c r="BF10" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="BG10">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="BH10">
         <v>0.24</v>
@@ -3959,7 +3959,7 @@
         <v>247</v>
       </c>
       <c r="BO10">
-        <v>104.8</v>
+        <v>112</v>
       </c>
       <c r="BP10">
         <v>5</v>
@@ -4132,7 +4132,7 @@
         <v>46.5</v>
       </c>
       <c r="BF11" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="BG11">
         <v>3.3</v>
@@ -4159,7 +4159,7 @@
         <v>248</v>
       </c>
       <c r="BO11">
-        <v>34</v>
+        <v>41.1</v>
       </c>
       <c r="BP11">
         <v>5</v>
@@ -4332,10 +4332,10 @@
         <v>75.7</v>
       </c>
       <c r="BF12" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="BG12">
-        <v>5.3</v>
+        <v>4.3</v>
       </c>
       <c r="BH12">
         <v>-0.27</v>
@@ -4359,7 +4359,7 @@
         <v>249</v>
       </c>
       <c r="BO12">
-        <v>204.5</v>
+        <v>211.6</v>
       </c>
       <c r="BP12">
         <v>5</v>
@@ -4532,10 +4532,10 @@
         <v>43.2</v>
       </c>
       <c r="BF13" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="BG13">
-        <v>2.7</v>
+        <v>3.1</v>
       </c>
       <c r="BH13">
         <v>-0.01</v>
@@ -4559,7 +4559,7 @@
         <v>250</v>
       </c>
       <c r="BO13">
-        <v>199</v>
+        <v>206.1</v>
       </c>
       <c r="BP13">
         <v>5</v>
@@ -4732,10 +4732,10 @@
         <v>24.4</v>
       </c>
       <c r="BF14" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="BG14">
-        <v>8.300000000000001</v>
+        <v>6.6</v>
       </c>
       <c r="BH14">
         <v>0.05</v>
@@ -4759,7 +4759,7 @@
         <v>251</v>
       </c>
       <c r="BO14">
-        <v>180.1</v>
+        <v>187.2</v>
       </c>
       <c r="BP14">
         <v>5</v>
@@ -4932,10 +4932,10 @@
         <v>76.90000000000001</v>
       </c>
       <c r="BF15" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="BG15">
-        <v>-2.4</v>
+        <v>-2.5</v>
       </c>
       <c r="BH15">
         <v>-0.25</v>
@@ -4959,7 +4959,7 @@
         <v>252</v>
       </c>
       <c r="BO15">
-        <v>91.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="BP15">
         <v>5</v>
@@ -5063,7 +5063,7 @@
         <v>2.4</v>
       </c>
       <c r="AI16">
-        <v>90.09999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="AJ16" t="s">
         <v>208</v>
@@ -5132,10 +5132,10 @@
         <v>72.7</v>
       </c>
       <c r="BF16" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="BG16">
-        <v>4.4</v>
+        <v>4</v>
       </c>
       <c r="BH16">
         <v>-0.25</v>
@@ -5159,7 +5159,7 @@
         <v>253</v>
       </c>
       <c r="BO16">
-        <v>199.8</v>
+        <v>206.9</v>
       </c>
       <c r="BP16">
         <v>5</v>
@@ -5332,10 +5332,10 @@
         <v>74.3</v>
       </c>
       <c r="BF17" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="BG17">
-        <v>-1.3</v>
+        <v>-1.5</v>
       </c>
       <c r="BH17">
         <v>0.77</v>
@@ -5359,7 +5359,7 @@
         <v>254</v>
       </c>
       <c r="BO17">
-        <v>65.7</v>
+        <v>72.8</v>
       </c>
       <c r="BP17">
         <v>5</v>
@@ -5926,7 +5926,7 @@
         <v>430</v>
       </c>
       <c r="J2">
-        <v>118.2</v>
+        <v>125.4</v>
       </c>
       <c r="K2">
         <v>0</v>
@@ -6318,7 +6318,7 @@
         <v>430</v>
       </c>
       <c r="J3">
-        <v>118.2</v>
+        <v>125.4</v>
       </c>
       <c r="K3">
         <v>0</v>
@@ -6710,7 +6710,7 @@
         <v>430</v>
       </c>
       <c r="J4">
-        <v>118.2</v>
+        <v>125.4</v>
       </c>
       <c r="K4">
         <v>0</v>
@@ -7102,7 +7102,7 @@
         <v>430</v>
       </c>
       <c r="J5">
-        <v>118.2</v>
+        <v>125.4</v>
       </c>
       <c r="K5">
         <v>0</v>
@@ -7494,10 +7494,10 @@
         <v>431</v>
       </c>
       <c r="J6">
-        <v>3.4</v>
+        <v>10.6</v>
       </c>
       <c r="K6">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L6">
         <v>5</v>
@@ -7886,10 +7886,10 @@
         <v>431</v>
       </c>
       <c r="J7">
-        <v>3.4</v>
+        <v>10.6</v>
       </c>
       <c r="K7">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="L7">
         <v>5</v>
@@ -8231,7 +8231,7 @@
         <v>235</v>
       </c>
       <c r="DU7">
-        <v>16.2</v>
+        <v>16.1</v>
       </c>
       <c r="DV7" t="s">
         <v>236</v>
@@ -8278,10 +8278,10 @@
         <v>431</v>
       </c>
       <c r="J8">
-        <v>3.4</v>
+        <v>10.6</v>
       </c>
       <c r="K8">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="L8">
         <v>5</v>
@@ -8670,10 +8670,10 @@
         <v>431</v>
       </c>
       <c r="J9">
-        <v>3.4</v>
+        <v>10.6</v>
       </c>
       <c r="K9">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="L9">
         <v>5</v>
@@ -9062,10 +9062,10 @@
         <v>432</v>
       </c>
       <c r="J10">
-        <v>95.5</v>
+        <v>102.7</v>
       </c>
       <c r="K10">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="L10">
         <v>5</v>
@@ -9454,10 +9454,10 @@
         <v>432</v>
       </c>
       <c r="J11">
-        <v>95.5</v>
+        <v>102.7</v>
       </c>
       <c r="K11">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="L11">
         <v>5</v>
@@ -9846,10 +9846,10 @@
         <v>432</v>
       </c>
       <c r="J12">
-        <v>95.5</v>
+        <v>102.7</v>
       </c>
       <c r="K12">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="L12">
         <v>5</v>
@@ -10238,10 +10238,10 @@
         <v>432</v>
       </c>
       <c r="J13">
-        <v>95.5</v>
+        <v>102.7</v>
       </c>
       <c r="K13">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="L13">
         <v>5</v>
@@ -10630,10 +10630,10 @@
         <v>433</v>
       </c>
       <c r="J14">
-        <v>78.5</v>
+        <v>85.7</v>
       </c>
       <c r="K14">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="L14">
         <v>5</v>
@@ -11022,10 +11022,10 @@
         <v>433</v>
       </c>
       <c r="J15">
-        <v>78.5</v>
+        <v>85.7</v>
       </c>
       <c r="K15">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="L15">
         <v>5</v>
@@ -11414,10 +11414,10 @@
         <v>433</v>
       </c>
       <c r="J16">
-        <v>78.5</v>
+        <v>85.7</v>
       </c>
       <c r="K16">
-        <v>3</v>
+        <v>2.9</v>
       </c>
       <c r="L16">
         <v>5</v>
@@ -11806,10 +11806,10 @@
         <v>433</v>
       </c>
       <c r="J17">
-        <v>78.5</v>
+        <v>85.7</v>
       </c>
       <c r="K17">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="L17">
         <v>5</v>
@@ -12198,10 +12198,10 @@
         <v>434</v>
       </c>
       <c r="J18">
-        <v>52.1</v>
+        <v>59.2</v>
       </c>
       <c r="K18">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="L18">
         <v>5</v>
@@ -12590,10 +12590,10 @@
         <v>434</v>
       </c>
       <c r="J19">
-        <v>52.1</v>
+        <v>59.2</v>
       </c>
       <c r="K19">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="L19">
         <v>5</v>
@@ -12982,10 +12982,10 @@
         <v>434</v>
       </c>
       <c r="J20">
-        <v>52.1</v>
+        <v>59.2</v>
       </c>
       <c r="K20">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="L20">
         <v>5</v>
@@ -13078,7 +13078,7 @@
         <v>5.7</v>
       </c>
       <c r="AP20">
-        <v>95.8</v>
+        <v>95.90000000000001</v>
       </c>
       <c r="AQ20">
         <v>56.7</v>
@@ -13374,10 +13374,10 @@
         <v>434</v>
       </c>
       <c r="J21">
-        <v>52.1</v>
+        <v>59.2</v>
       </c>
       <c r="K21">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="L21">
         <v>5</v>
@@ -13766,10 +13766,10 @@
         <v>435</v>
       </c>
       <c r="J22">
-        <v>205.7</v>
+        <v>212.9</v>
       </c>
       <c r="K22">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="L22">
         <v>5</v>
@@ -14158,10 +14158,10 @@
         <v>435</v>
       </c>
       <c r="J23">
-        <v>205.7</v>
+        <v>212.9</v>
       </c>
       <c r="K23">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="L23">
         <v>5</v>
@@ -14550,10 +14550,10 @@
         <v>435</v>
       </c>
       <c r="J24">
-        <v>205.7</v>
+        <v>212.9</v>
       </c>
       <c r="K24">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="L24">
         <v>5</v>
@@ -14942,10 +14942,10 @@
         <v>435</v>
       </c>
       <c r="J25">
-        <v>205.7</v>
+        <v>212.9</v>
       </c>
       <c r="K25">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="L25">
         <v>5</v>
@@ -15334,10 +15334,10 @@
         <v>436</v>
       </c>
       <c r="J26">
-        <v>104.2</v>
+        <v>111.4</v>
       </c>
       <c r="K26">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="L26">
         <v>5</v>
@@ -15726,10 +15726,10 @@
         <v>436</v>
       </c>
       <c r="J27">
-        <v>104.2</v>
+        <v>111.4</v>
       </c>
       <c r="K27">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="L27">
         <v>5</v>
@@ -16118,10 +16118,10 @@
         <v>436</v>
       </c>
       <c r="J28">
-        <v>104.2</v>
+        <v>111.4</v>
       </c>
       <c r="K28">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="L28">
         <v>5</v>
@@ -16510,10 +16510,10 @@
         <v>436</v>
       </c>
       <c r="J29">
-        <v>104.2</v>
+        <v>111.4</v>
       </c>
       <c r="K29">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="L29">
         <v>5</v>
@@ -16902,10 +16902,10 @@
         <v>430</v>
       </c>
       <c r="J30">
-        <v>118.9</v>
+        <v>126</v>
       </c>
       <c r="K30">
-        <v>1.5</v>
+        <v>1.4</v>
       </c>
       <c r="L30">
         <v>5</v>
@@ -17294,10 +17294,10 @@
         <v>430</v>
       </c>
       <c r="J31">
-        <v>118.9</v>
+        <v>126</v>
       </c>
       <c r="K31">
-        <v>2.5</v>
+        <v>2.4</v>
       </c>
       <c r="L31">
         <v>5</v>
@@ -17686,10 +17686,10 @@
         <v>430</v>
       </c>
       <c r="J32">
-        <v>118.9</v>
+        <v>126</v>
       </c>
       <c r="K32">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
       <c r="L32">
         <v>5</v>
@@ -18078,10 +18078,10 @@
         <v>430</v>
       </c>
       <c r="J33">
-        <v>118.9</v>
+        <v>126</v>
       </c>
       <c r="K33">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="L33">
         <v>5</v>
@@ -18470,10 +18470,10 @@
         <v>437</v>
       </c>
       <c r="J34">
-        <v>104.8</v>
+        <v>112</v>
       </c>
       <c r="K34">
-        <v>1.9</v>
+        <v>1.8</v>
       </c>
       <c r="L34">
         <v>5</v>
@@ -18862,10 +18862,10 @@
         <v>437</v>
       </c>
       <c r="J35">
-        <v>104.8</v>
+        <v>112</v>
       </c>
       <c r="K35">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="L35">
         <v>5</v>
@@ -19254,10 +19254,10 @@
         <v>437</v>
       </c>
       <c r="J36">
-        <v>104.8</v>
+        <v>112</v>
       </c>
       <c r="K36">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="L36">
         <v>5</v>
@@ -19350,7 +19350,7 @@
         <v>16.2</v>
       </c>
       <c r="AP36">
-        <v>89.90000000000001</v>
+        <v>90</v>
       </c>
       <c r="AQ36">
         <v>68.59999999999999</v>
@@ -19646,10 +19646,10 @@
         <v>437</v>
       </c>
       <c r="J37">
-        <v>104.8</v>
+        <v>112</v>
       </c>
       <c r="K37">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="L37">
         <v>5</v>
@@ -20038,10 +20038,10 @@
         <v>438</v>
       </c>
       <c r="J38">
-        <v>34</v>
+        <v>41.1</v>
       </c>
       <c r="K38">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="L38">
         <v>5</v>
@@ -20374,7 +20374,7 @@
         <v>237</v>
       </c>
       <c r="DU38">
-        <v>3.6</v>
+        <v>3.5</v>
       </c>
       <c r="DV38" t="s">
         <v>236</v>
@@ -20421,10 +20421,10 @@
         <v>438</v>
       </c>
       <c r="J39">
-        <v>34</v>
+        <v>41.1</v>
       </c>
       <c r="K39">
-        <v>3.3</v>
+        <v>3.2</v>
       </c>
       <c r="L39">
         <v>5</v>
@@ -20804,10 +20804,10 @@
         <v>438</v>
       </c>
       <c r="J40">
-        <v>34</v>
+        <v>41.1</v>
       </c>
       <c r="K40">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="L40">
         <v>5</v>
@@ -21187,10 +21187,10 @@
         <v>438</v>
       </c>
       <c r="J41">
-        <v>34</v>
+        <v>41.1</v>
       </c>
       <c r="K41">
-        <v>5.3</v>
+        <v>5.2</v>
       </c>
       <c r="L41">
         <v>5</v>
@@ -21570,10 +21570,10 @@
         <v>439</v>
       </c>
       <c r="J42">
-        <v>204.5</v>
+        <v>211.6</v>
       </c>
       <c r="K42">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="L42">
         <v>5</v>
@@ -21962,10 +21962,10 @@
         <v>439</v>
       </c>
       <c r="J43">
-        <v>204.5</v>
+        <v>211.6</v>
       </c>
       <c r="K43">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="L43">
         <v>5</v>
@@ -22307,7 +22307,7 @@
         <v>235</v>
       </c>
       <c r="DU43">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="DV43" t="s">
         <v>236</v>
@@ -22354,10 +22354,10 @@
         <v>439</v>
       </c>
       <c r="J44">
-        <v>204.5</v>
+        <v>211.6</v>
       </c>
       <c r="K44">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="L44">
         <v>5</v>
@@ -22699,7 +22699,7 @@
         <v>236</v>
       </c>
       <c r="DU44">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="DV44" t="s">
         <v>236</v>
@@ -22746,10 +22746,10 @@
         <v>439</v>
       </c>
       <c r="J45">
-        <v>204.5</v>
+        <v>211.6</v>
       </c>
       <c r="K45">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="L45">
         <v>5</v>
@@ -23138,10 +23138,10 @@
         <v>440</v>
       </c>
       <c r="J46">
-        <v>199</v>
+        <v>206.1</v>
       </c>
       <c r="K46">
-        <v>2.4</v>
+        <v>2.3</v>
       </c>
       <c r="L46">
         <v>5</v>
@@ -23234,7 +23234,7 @@
         <v>4.6</v>
       </c>
       <c r="AP46">
-        <v>96</v>
+        <v>96.09999999999999</v>
       </c>
       <c r="AQ46">
         <v>73.09999999999999</v>
@@ -23530,10 +23530,10 @@
         <v>440</v>
       </c>
       <c r="J47">
-        <v>199</v>
+        <v>206.1</v>
       </c>
       <c r="K47">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="L47">
         <v>5</v>
@@ -23626,7 +23626,7 @@
         <v>4.9</v>
       </c>
       <c r="AP47">
-        <v>96.59999999999999</v>
+        <v>96.7</v>
       </c>
       <c r="AQ47">
         <v>68.90000000000001</v>
@@ -23922,10 +23922,10 @@
         <v>440</v>
       </c>
       <c r="J48">
-        <v>199</v>
+        <v>206.1</v>
       </c>
       <c r="K48">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="L48">
         <v>5</v>
@@ -24314,10 +24314,10 @@
         <v>440</v>
       </c>
       <c r="J49">
-        <v>199</v>
+        <v>206.1</v>
       </c>
       <c r="K49">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="L49">
         <v>5</v>
@@ -24706,10 +24706,10 @@
         <v>441</v>
       </c>
       <c r="J50">
-        <v>180.1</v>
+        <v>187.2</v>
       </c>
       <c r="K50">
-        <v>2.9</v>
+        <v>2.8</v>
       </c>
       <c r="L50">
         <v>5</v>
@@ -24802,7 +24802,7 @@
         <v>10.4</v>
       </c>
       <c r="AP50">
-        <v>91</v>
+        <v>91.09999999999999</v>
       </c>
       <c r="AQ50">
         <v>74.5</v>
@@ -25098,10 +25098,10 @@
         <v>441</v>
       </c>
       <c r="J51">
-        <v>180.1</v>
+        <v>187.2</v>
       </c>
       <c r="K51">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="L51">
         <v>5</v>
@@ -25197,7 +25197,7 @@
         <v>86.59999999999999</v>
       </c>
       <c r="AQ51">
-        <v>78.5</v>
+        <v>78.59999999999999</v>
       </c>
       <c r="AR51">
         <v>1.05</v>
@@ -25490,10 +25490,10 @@
         <v>441</v>
       </c>
       <c r="J52">
-        <v>180.1</v>
+        <v>187.2</v>
       </c>
       <c r="K52">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="L52">
         <v>5</v>
@@ -25882,10 +25882,10 @@
         <v>441</v>
       </c>
       <c r="J53">
-        <v>180.1</v>
+        <v>187.2</v>
       </c>
       <c r="K53">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="L53">
         <v>5</v>
@@ -26274,10 +26274,10 @@
         <v>442</v>
       </c>
       <c r="J54">
-        <v>91.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="K54">
-        <v>3.9</v>
+        <v>3.8</v>
       </c>
       <c r="L54">
         <v>5</v>
@@ -26619,7 +26619,7 @@
         <v>236</v>
       </c>
       <c r="DU54">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="DV54" t="s">
         <v>236</v>
@@ -26666,10 +26666,10 @@
         <v>442</v>
       </c>
       <c r="J55">
-        <v>91.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="K55">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="L55">
         <v>5</v>
@@ -27058,10 +27058,10 @@
         <v>442</v>
       </c>
       <c r="J56">
-        <v>91.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="K56">
-        <v>5.9</v>
+        <v>5.8</v>
       </c>
       <c r="L56">
         <v>5</v>
@@ -27450,10 +27450,10 @@
         <v>442</v>
       </c>
       <c r="J57">
-        <v>91.09999999999999</v>
+        <v>98.2</v>
       </c>
       <c r="K57">
-        <v>6.9</v>
+        <v>6.8</v>
       </c>
       <c r="L57">
         <v>5</v>
@@ -27842,10 +27842,10 @@
         <v>443</v>
       </c>
       <c r="J58">
-        <v>199.8</v>
+        <v>206.9</v>
       </c>
       <c r="K58">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="L58">
         <v>5</v>
@@ -28234,10 +28234,10 @@
         <v>443</v>
       </c>
       <c r="J59">
-        <v>199.8</v>
+        <v>206.9</v>
       </c>
       <c r="K59">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="L59">
         <v>5</v>
@@ -28626,10 +28626,10 @@
         <v>443</v>
       </c>
       <c r="J60">
-        <v>199.8</v>
+        <v>206.9</v>
       </c>
       <c r="K60">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="L60">
         <v>5</v>
@@ -29018,10 +29018,10 @@
         <v>443</v>
       </c>
       <c r="J61">
-        <v>199.8</v>
+        <v>206.9</v>
       </c>
       <c r="K61">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="L61">
         <v>5</v>
@@ -29114,7 +29114,7 @@
         <v>15</v>
       </c>
       <c r="AP61">
-        <v>86.3</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="AQ61">
         <v>57.7</v>
@@ -29363,7 +29363,7 @@
         <v>236</v>
       </c>
       <c r="DU61">
-        <v>12.6</v>
+        <v>12.5</v>
       </c>
       <c r="DV61" t="s">
         <v>236</v>
@@ -29410,10 +29410,10 @@
         <v>444</v>
       </c>
       <c r="J62">
-        <v>65.7</v>
+        <v>72.8</v>
       </c>
       <c r="K62">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="L62">
         <v>5</v>
@@ -29802,10 +29802,10 @@
         <v>444</v>
       </c>
       <c r="J63">
-        <v>65.7</v>
+        <v>72.8</v>
       </c>
       <c r="K63">
-        <v>5.4</v>
+        <v>5.3</v>
       </c>
       <c r="L63">
         <v>5</v>
@@ -30194,10 +30194,10 @@
         <v>444</v>
       </c>
       <c r="J64">
-        <v>65.7</v>
+        <v>72.8</v>
       </c>
       <c r="K64">
-        <v>6.4</v>
+        <v>6.3</v>
       </c>
       <c r="L64">
         <v>5</v>
@@ -30586,10 +30586,10 @@
         <v>444</v>
       </c>
       <c r="J65">
-        <v>65.7</v>
+        <v>72.8</v>
       </c>
       <c r="K65">
-        <v>7.4</v>
+        <v>7.3</v>
       </c>
       <c r="L65">
         <v>5</v>
@@ -31372,7 +31372,7 @@
         <v>189</v>
       </c>
       <c r="G8">
-        <v>90.09999999999999</v>
+        <v>90.2</v>
       </c>
       <c r="H8">
         <v>5</v>

</xml_diff>